<commit_message>
Cria estrutura inicial das abas do sistema financeiro
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -1,13 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B7EA02-39E1-424E-951E-527C3588729F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Plan1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
+    <sheet name="Resumo_Mensal" sheetId="3" r:id="rId2"/>
+    <sheet name="Receitas" sheetId="4" r:id="rId3"/>
+    <sheet name="Despesas" sheetId="5" r:id="rId4"/>
+    <sheet name="Cartoes" sheetId="6" r:id="rId5"/>
+    <sheet name="Parcelamentos" sheetId="7" r:id="rId6"/>
+    <sheet name="Investimentos" sheetId="8" r:id="rId7"/>
+    <sheet name="Contas_Bancarias" sheetId="9" r:id="rId8"/>
+    <sheet name="Patrimonio" sheetId="10" r:id="rId9"/>
+    <sheet name="Metas" sheetId="11" r:id="rId10"/>
+    <sheet name="Historico" sheetId="12" r:id="rId11"/>
+    <sheet name="Listas" sheetId="13" r:id="rId12"/>
+    <sheet name="Configuracoes" sheetId="14" r:id="rId13"/>
+    <sheet name="Calculos" sheetId="15" r:id="rId14"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -19,7 +38,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -330,10 +349,127 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43B9CDE1-C651-4C54-846A-6054721D80A4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1823272F-9888-4754-9B1E-EFD816629FC8}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25ADEA5B-E592-467E-96CE-CA4251B085F7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF8BB2A8-B031-40A7-9D90-72F49B830BAB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FC72ED-E857-46F3-96F1-3B41006EF91A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90BE9016-E170-4996-8755-6189BC2FB397}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498502DD-C545-4B1D-ABFA-496F14762B9E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B78059A9-CFA8-4DFA-9FD1-F4F4F098960D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50634029-1690-41A0-83DB-813CACF2A824}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28EAEDA-7868-4003-99EF-6D6DDD98D4D1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95784DD6-1DE2-4B31-9DA2-D36FD96B3EE9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93542742-5C03-4631-B7AD-2B736A5A5239}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F16A19F-C13A-4E89-BB61-B22C4601171D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Cria listas de apoio do sistema financeiro
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B7EA02-39E1-424E-951E-527C3588729F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0292A1E6-7F2D-4691-84E2-D3942469F8AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="6" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -37,10 +37,101 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+  <si>
+    <t>Tipos_Receita</t>
+  </si>
+  <si>
+    <t>Salario</t>
+  </si>
+  <si>
+    <t>Bonus</t>
+  </si>
+  <si>
+    <t>Investimentos</t>
+  </si>
+  <si>
+    <t>Outros</t>
+  </si>
+  <si>
+    <t>Tipos_Despesa</t>
+  </si>
+  <si>
+    <t>Moradia</t>
+  </si>
+  <si>
+    <t>Alimentacao</t>
+  </si>
+  <si>
+    <t>Transporte</t>
+  </si>
+  <si>
+    <t>Saude</t>
+  </si>
+  <si>
+    <t>Educacao</t>
+  </si>
+  <si>
+    <t>Lazer</t>
+  </si>
+  <si>
+    <t>Formas_Pagamento</t>
+  </si>
+  <si>
+    <t>Dinheiro</t>
+  </si>
+  <si>
+    <t>Pix</t>
+  </si>
+  <si>
+    <t>Cartao</t>
+  </si>
+  <si>
+    <t>Debito</t>
+  </si>
+  <si>
+    <t>Transferencia</t>
+  </si>
+  <si>
+    <t>Contas_Bancarias</t>
+  </si>
+  <si>
+    <t>Nubank</t>
+  </si>
+  <si>
+    <t>Banco_Inter</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Pago</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
+    <t>Ativo</t>
+  </si>
+  <si>
+    <t>Concluido</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -68,8 +159,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -377,10 +470,122 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25ADEA5B-E592-467E-96CE-CA4251B085F7}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="9" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2"/>
+      <c r="E1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" s="2"/>
+      <c r="G1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="2"/>
+      <c r="I1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>4</v>
+      </c>
+      <c r="I5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Finaliza estrutura da aba Receitas
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0292A1E6-7F2D-4691-84E2-D3942469F8AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F427901-1CB9-4C1F-93F5-B6941104DC71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="6" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,11 @@
     <sheet name="Configuracoes" sheetId="14" r:id="rId13"/>
     <sheet name="Calculos" sheetId="15" r:id="rId14"/>
   </sheets>
+  <definedNames>
+    <definedName name="lstContasBancarias">Listas!$G$2:$G$5</definedName>
+    <definedName name="lstStatus">Listas!$I$2:$I$5</definedName>
+    <definedName name="lstTiposReceita">Listas!$A$2:$A$5</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -116,13 +121,40 @@
   </si>
   <si>
     <t>Concluido</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Descricao</t>
+  </si>
+  <si>
+    <t>Tipo_Receita</t>
+  </si>
+  <si>
+    <t>Valor</t>
+  </si>
+  <si>
+    <t>Conta_Bancaria</t>
+  </si>
+  <si>
+    <t>Observacao</t>
+  </si>
+  <si>
+    <t>Salario Julho</t>
+  </si>
+  <si>
+    <t>Salario CLT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,6 +164,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -156,15 +195,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -178,6 +220,22 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{55300694-91AF-4EEF-A885-E13BA79E50C1}" name="tbReceitas" displayName="tbReceitas" ref="A1:G2" totalsRowShown="0">
+  <autoFilter ref="A1:G2" xr:uid="{55300694-91AF-4EEF-A885-E13BA79E50C1}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{813C2834-4B6B-482C-AB37-6B8EA07A07D4}" name="Data"/>
+    <tableColumn id="2" xr3:uid="{699720BF-24C2-46BE-A82A-B5C5965F6CFB}" name="Descricao"/>
+    <tableColumn id="3" xr3:uid="{B8B413D5-A000-49D6-85F5-1A691E4531A9}" name="Tipo_Receita"/>
+    <tableColumn id="4" xr3:uid="{F5150B90-B4BA-410F-A636-FF84688F78C2}" name="Valor" dataCellStyle="Moeda"/>
+    <tableColumn id="5" xr3:uid="{27840D25-3EEA-4664-89C1-FDC8C605AE0D}" name="Conta_Bancaria"/>
+    <tableColumn id="6" xr3:uid="{9C7B06CE-235C-4065-8819-0BA072F8473F}" name="Observacao"/>
+    <tableColumn id="7" xr3:uid="{5E447685-E5DD-4C17-9D8B-4ADA1892F798}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -480,19 +538,15 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
       <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2"/>
       <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="2"/>
       <c r="G1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="2"/>
       <c r="I1" s="1" t="s">
         <v>21</v>
       </c>
@@ -618,10 +672,81 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498502DD-C545-4B1D-ABFA-496F14762B9E}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <dimension ref="A1:G2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46208</v>
+      </c>
+      <c r="B2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>2700</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2" xr:uid="{5030F56A-771B-4A5F-80B1-5FCE33DCCABF}">
+      <formula1>lstTiposReceita</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{5305F043-02F9-4FFE-AE21-7A516EB9ACAE}">
+      <formula1>lstContasBancarias</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{962BDD76-CAEE-4C6C-9D99-EC80B8F368C1}">
+      <formula1>lstStatus</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Cria estrutura da aba Despesas
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F427901-1CB9-4C1F-93F5-B6941104DC71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5661254C-27B7-48D8-90D0-BE8766BD7DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,7 @@
   <definedNames>
     <definedName name="lstContasBancarias">Listas!$G$2:$G$5</definedName>
     <definedName name="lstStatus">Listas!$I$2:$I$5</definedName>
+    <definedName name="lstTiposDespesa">Listas!$C$2:$C$8</definedName>
     <definedName name="lstTiposReceita">Listas!$A$2:$A$5</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="37">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -145,6 +146,15 @@
   </si>
   <si>
     <t>Salario CLT</t>
+  </si>
+  <si>
+    <t>Tipo_Despesa</t>
+  </si>
+  <si>
+    <t>teste</t>
+  </si>
+  <si>
+    <t>Teste de sistema</t>
   </si>
 </sst>
 </file>
@@ -209,7 +219,11 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -233,6 +247,22 @@
     <tableColumn id="5" xr3:uid="{27840D25-3EEA-4664-89C1-FDC8C605AE0D}" name="Conta_Bancaria"/>
     <tableColumn id="6" xr3:uid="{9C7B06CE-235C-4065-8819-0BA072F8473F}" name="Observacao"/>
     <tableColumn id="7" xr3:uid="{5E447685-E5DD-4C17-9D8B-4ADA1892F798}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E324B775-B412-4705-AA40-FE3CDCC0BA58}" name="tbDespesas" displayName="tbDespesas" ref="A1:G3" totalsRowShown="0">
+  <autoFilter ref="A1:G3" xr:uid="{E324B775-B412-4705-AA40-FE3CDCC0BA58}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{348CBD6E-BAB2-4453-B3DB-59361AD0A0F2}" name="Data" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{A4C6D8F4-18F9-4E8D-A471-DAA5D2F84E4D}" name="Descricao"/>
+    <tableColumn id="3" xr3:uid="{0EF10707-0FC4-4B03-ADA9-20680CA6C867}" name="Tipo_Despesa"/>
+    <tableColumn id="4" xr3:uid="{6FE19F1B-8AC6-480C-BBD0-6B739B3F311C}" name="Valor" dataCellStyle="Moeda"/>
+    <tableColumn id="5" xr3:uid="{4C7BEAE2-AA61-4167-96A8-B13319F12C81}" name="Conta_Bancaria"/>
+    <tableColumn id="6" xr3:uid="{20E14D20-80B3-4C18-B94B-5DA351060A83}" name="Observacao"/>
+    <tableColumn id="7" xr3:uid="{61E2C68E-F125-44C4-8AA8-2FDA95423A81}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -752,10 +782,85 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B78059A9-CFA8-4DFA-9FD1-F4F4F098960D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46216</v>
+      </c>
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="3">
+        <v>50</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="D3" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C3" xr:uid="{966CA5DC-7167-4F11-A88D-7BD00A6D67A6}">
+      <formula1>lstTiposDespesa</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E3" xr:uid="{42027A5D-3623-4F73-A193-79875C7B49CD}">
+      <formula1>lstContasBancarias</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G3" xr:uid="{2C82B0D7-FC1E-4875-B666-56F46C3F3BE2}">
+      <formula1>lstStatus</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Cria módulo de configurações do sistema
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36535C6F-CADB-4586-9E51-70CA64C4C7F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A2ABF4-F9F4-4FCB-8C27-5A2540A193AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="7" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,19 @@
     <definedName name="NomeSistema">Configuracoes!$B$2</definedName>
     <definedName name="VersaoSistema">Configuracoes!$B$3</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -573,9 +582,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="str">
+        <f>NomeSistema</f>
+        <v>Sistema Financeiro Carlos</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>VersaoSistema</f>
+        <v>1.0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Cria indicadores iniciais do Dashboard
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A2ABF4-F9F4-4FCB-8C27-5A2540A193AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF4B957-3A74-41CA-92FD-28E77A3F2835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -192,6 +192,15 @@
   </si>
   <si>
     <t>Ano_Inicial</t>
+  </si>
+  <si>
+    <t>Total de Receitas</t>
+  </si>
+  <si>
+    <t>Total de Despesas</t>
+  </si>
+  <si>
+    <t>Saldo Atual</t>
   </si>
 </sst>
 </file>
@@ -582,23 +591,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="str">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="str">
         <f>NomeSistema</f>
         <v>Sistema Financeiro Carlos</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="str">
-        <f>VersaoSistema</f>
-        <v>1.0</v>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="str">
+        <f>"Versão "&amp;VersaoSistema</f>
+        <v>Versão 1.0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="str">
+        <f>"Ano de referência: "&amp;AnoInicial</f>
+        <v>Ano de referência: 2026</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="3">
+        <f>SUM(tbReceitas[Valor])</f>
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="3">
+        <f>SUM(tbDespesas[Valor])</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="3">
+        <f>B5-B6</f>
+        <v>2650</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Cria resumo mensal com cálculos de receitas e despesas
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF4B957-3A74-41CA-92FD-28E77A3F2835}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CDC6DD7-371A-43E5-A19A-F940C18F2C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -201,6 +201,21 @@
   </si>
   <si>
     <t>Saldo Atual</t>
+  </si>
+  <si>
+    <t>Mes</t>
+  </si>
+  <si>
+    <t>Ano</t>
+  </si>
+  <si>
+    <t>Total_Receitas</t>
+  </si>
+  <si>
+    <t>Total_Despesas</t>
+  </si>
+  <si>
+    <t>Saldo</t>
   </si>
 </sst>
 </file>
@@ -286,6 +301,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8A0F6549-5E43-427D-967B-3F5766F66080}" name="tbResumoMensal" displayName="tbResumoMensal" ref="A1:E2" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{8A0F6549-5E43-427D-967B-3F5766F66080}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{3AF8D024-BA06-435E-AA5D-554538ED1BB5}" name="Mes"/>
+    <tableColumn id="2" xr3:uid="{352D13CF-CC82-4D16-890B-7CFCBF56C180}" name="Ano"/>
+    <tableColumn id="3" xr3:uid="{F285CC66-5EAA-49D5-B5B4-EB5FE193323D}" name="Total_Receitas" dataCellStyle="Moeda">
+      <calculatedColumnFormula>SUMIFS(tbReceitas[Valor],tbReceitas[Data],"&gt;="&amp;DATE(B2,A2,1),tbReceitas[Data],"&lt;"&amp;DATE(B2,A2+1,1))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{053912A3-621A-4F93-A624-907418D8D463}" name="Total_Despesas" dataCellStyle="Moeda"/>
+    <tableColumn id="5" xr3:uid="{255444C8-9635-4814-BE21-BFC9913BD2EF}" name="Saldo" dataCellStyle="Moeda">
+      <calculatedColumnFormula>C2-D2</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{55300694-91AF-4EEF-A885-E13BA79E50C1}" name="tbReceitas" displayName="tbReceitas" ref="A1:G2" totalsRowShown="0">
   <autoFilter ref="A1:G2" xr:uid="{55300694-91AF-4EEF-A885-E13BA79E50C1}"/>
   <tableColumns count="7">
@@ -301,7 +334,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{E324B775-B412-4705-AA40-FE3CDCC0BA58}" name="tbDespesas" displayName="tbDespesas" ref="A1:G3" totalsRowShown="0">
   <autoFilter ref="A1:G3" xr:uid="{E324B775-B412-4705-AA40-FE3CDCC0BA58}"/>
   <tableColumns count="7">
@@ -317,7 +350,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}" name="tbConfiguracoes" displayName="tbConfiguracoes" ref="A1:B5" totalsRowShown="0">
   <autoFilter ref="A1:B5" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}"/>
   <tableColumns count="2">
@@ -852,10 +885,57 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90BE9016-E170-4996-8755-6189BC2FB397}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="2" width="6.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>2026</v>
+      </c>
+      <c r="C2" s="3">
+        <f>SUMIFS(tbReceitas[Valor],tbReceitas[Data],"&gt;="&amp;DATE(B2,A2,1),tbReceitas[Data],"&lt;"&amp;DATE(B2,A2+1,1))</f>
+        <v>2700</v>
+      </c>
+      <c r="D2" s="3">
+        <v>50</v>
+      </c>
+      <c r="E2" s="3">
+        <f>C2-D2</f>
+        <v>2650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Conecta Dashboard ao resumo mensal
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CDC6DD7-371A-43E5-A19A-F940C18F2C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4447A24B-DFFC-4E7A-8308-1613EE95C077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -29,11 +29,13 @@
     <sheet name="Calculos" sheetId="15" r:id="rId14"/>
   </sheets>
   <definedNames>
+    <definedName name="AnoAnalise">Configuracoes!$B$7</definedName>
     <definedName name="AnoInicial">Configuracoes!$B$5</definedName>
     <definedName name="lstContasBancarias">Listas!$G$2:$G$5</definedName>
     <definedName name="lstStatus">Listas!$I$2:$I$5</definedName>
     <definedName name="lstTiposDespesa">Listas!$C$2:$C$8</definedName>
     <definedName name="lstTiposReceita">Listas!$A$2:$A$5</definedName>
+    <definedName name="MesAnalise">Configuracoes!$B$6</definedName>
     <definedName name="MoedaSistema">Configuracoes!$B$4</definedName>
     <definedName name="NomeSistema">Configuracoes!$B$2</definedName>
     <definedName name="VersaoSistema">Configuracoes!$B$3</definedName>
@@ -56,8 +58,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -216,6 +240,12 @@
   </si>
   <si>
     <t>Saldo</t>
+  </si>
+  <si>
+    <t>MesAnalise</t>
+  </si>
+  <si>
+    <t>AnoAnalise</t>
   </si>
 </sst>
 </file>
@@ -304,8 +334,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{8A0F6549-5E43-427D-967B-3F5766F66080}" name="tbResumoMensal" displayName="tbResumoMensal" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{8A0F6549-5E43-427D-967B-3F5766F66080}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{3AF8D024-BA06-435E-AA5D-554538ED1BB5}" name="Mes"/>
-    <tableColumn id="2" xr3:uid="{352D13CF-CC82-4D16-890B-7CFCBF56C180}" name="Ano"/>
+    <tableColumn id="1" xr3:uid="{3AF8D024-BA06-435E-AA5D-554538ED1BB5}" name="Mes">
+      <calculatedColumnFormula>MesAnalise</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{352D13CF-CC82-4D16-890B-7CFCBF56C180}" name="Ano">
+      <calculatedColumnFormula>AnoAnalise</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="3" xr3:uid="{F285CC66-5EAA-49D5-B5B4-EB5FE193323D}" name="Total_Receitas" dataCellStyle="Moeda">
       <calculatedColumnFormula>SUMIFS(tbReceitas[Valor],tbReceitas[Data],"&gt;="&amp;DATE(B2,A2,1),tbReceitas[Data],"&lt;"&amp;DATE(B2,A2+1,1))</calculatedColumnFormula>
     </tableColumn>
@@ -351,8 +385,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}" name="tbConfiguracoes" displayName="tbConfiguracoes" ref="A1:B5" totalsRowShown="0">
-  <autoFilter ref="A1:B5" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}" name="tbConfiguracoes" displayName="tbConfiguracoes" ref="A1:B7" totalsRowShown="0">
+  <autoFilter ref="A1:B7" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D2936EAB-86F0-4B66-ACE9-63DAD986A44F}" name="Parametro"/>
     <tableColumn id="2" xr3:uid="{F4458E02-E9B4-48E4-A708-C914B6098752}" name="Valor"/>
@@ -653,8 +687,8 @@
       <c r="A5" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="3">
-        <f>SUM(tbReceitas[Valor])</f>
+      <c r="B5" s="3" cm="1">
+        <f t="array" ref="B5">tbResumoMensal[Total_Receitas]</f>
         <v>2700</v>
       </c>
     </row>
@@ -662,8 +696,8 @@
       <c r="A6" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="3">
-        <f>SUM(tbDespesas[Valor])</f>
+      <c r="B6" s="3" cm="1">
+        <f t="array" ref="B6">tbResumoMensal[Total_Despesas]</f>
         <v>50</v>
       </c>
     </row>
@@ -671,8 +705,8 @@
       <c r="A7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="3">
-        <f>B5-B6</f>
+      <c r="B7" s="3" cm="1">
+        <f t="array" ref="B7">tbResumoMensal[Saldo]</f>
         <v>2650</v>
       </c>
     </row>
@@ -819,7 +853,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF8BB2A8-B031-40A7-9D90-72F49B830BAB}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
@@ -863,6 +897,22 @@
         <v>44</v>
       </c>
       <c r="B5" s="4">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="4">
         <v>2026</v>
       </c>
     </row>
@@ -914,9 +964,11 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
+        <f>MesAnalise</f>
         <v>7</v>
       </c>
       <c r="B2">
+        <f>AnoAnalise</f>
         <v>2026</v>
       </c>
       <c r="C2" s="3">

</xml_diff>

<commit_message>
Cria estrutura inicial de cartões e parcelamentos
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4447A24B-DFFC-4E7A-8308-1613EE95C077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FEC1B3-8803-45FF-A9FA-4BC6FFF63069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -27,10 +27,15 @@
     <sheet name="Listas" sheetId="13" r:id="rId12"/>
     <sheet name="Configuracoes" sheetId="14" r:id="rId13"/>
     <sheet name="Calculos" sheetId="15" r:id="rId14"/>
+    <sheet name="Faturas" sheetId="17" r:id="rId15"/>
+    <sheet name="Lancamentos_Cartao" sheetId="18" r:id="rId16"/>
+    <sheet name="," sheetId="19" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="AnoAnalise">Configuracoes!$B$7</definedName>
     <definedName name="AnoInicial">Configuracoes!$B$5</definedName>
+    <definedName name="lstCartoes">tbCartoes[Nome_Cartao]</definedName>
+    <definedName name="lstCategoriasCartao">Listas!$K$2:$K$7</definedName>
     <definedName name="lstContasBancarias">Listas!$G$2:$G$5</definedName>
     <definedName name="lstStatus">Listas!$I$2:$I$5</definedName>
     <definedName name="lstTiposDespesa">Listas!$C$2:$C$8</definedName>
@@ -59,7 +64,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -81,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="83">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -246,6 +251,90 @@
   </si>
   <si>
     <t>AnoAnalise</t>
+  </si>
+  <si>
+    <t>Nome_Cartao</t>
+  </si>
+  <si>
+    <t>Banco</t>
+  </si>
+  <si>
+    <t>Limite</t>
+  </si>
+  <si>
+    <t>Dia_Fechamento</t>
+  </si>
+  <si>
+    <t>Dia_Vencimento</t>
+  </si>
+  <si>
+    <t>Atacadao</t>
+  </si>
+  <si>
+    <t>Banco_Atacadao</t>
+  </si>
+  <si>
+    <t>Inter</t>
+  </si>
+  <si>
+    <t>Banco_Nubank</t>
+  </si>
+  <si>
+    <t>Carrefour</t>
+  </si>
+  <si>
+    <t>Banco_Carrefour</t>
+  </si>
+  <si>
+    <t>Competencia</t>
+  </si>
+  <si>
+    <t>Data_Vencimento</t>
+  </si>
+  <si>
+    <t>Valor_Fatura</t>
+  </si>
+  <si>
+    <t>Status_Pagamento</t>
+  </si>
+  <si>
+    <t>Data_Compra</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Parcelas</t>
+  </si>
+  <si>
+    <t>Categoria_Cartao</t>
+  </si>
+  <si>
+    <t>Mercado</t>
+  </si>
+  <si>
+    <t>Combustivel</t>
+  </si>
+  <si>
+    <t>Compras</t>
+  </si>
+  <si>
+    <t>Assinaturas</t>
+  </si>
+  <si>
+    <t>Notebook</t>
+  </si>
+  <si>
+    <t>Compra</t>
+  </si>
+  <si>
+    <t>Parcela_Atual</t>
+  </si>
+  <si>
+    <t>Total_Parcelas</t>
+  </si>
+  <si>
+    <t>Valor_Parcela</t>
   </si>
 </sst>
 </file>
@@ -300,7 +389,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -308,6 +397,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -385,11 +475,74 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{8B65EBCC-D5C1-48BD-B7A7-BC0389AC0DBC}" name="tbCartoes" displayName="tbCartoes" ref="A1:F5" totalsRowShown="0">
+  <autoFilter ref="A1:F5" xr:uid="{8B65EBCC-D5C1-48BD-B7A7-BC0389AC0DBC}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{7F7848B9-A0F0-4055-BB04-6D5C7EF9CBEC}" name="Nome_Cartao"/>
+    <tableColumn id="2" xr3:uid="{2D95D798-8C82-4869-8800-04F0EB9593F3}" name="Banco"/>
+    <tableColumn id="3" xr3:uid="{5579189E-E0FE-4458-85CD-FFE6AC91E1AF}" name="Limite" dataCellStyle="Moeda"/>
+    <tableColumn id="4" xr3:uid="{4746A5F2-D538-4B68-9653-3DA7B5DB7104}" name="Dia_Fechamento"/>
+    <tableColumn id="5" xr3:uid="{D9D3B0A1-24C6-4B02-97DC-553E425AC7A6}" name="Dia_Vencimento"/>
+    <tableColumn id="6" xr3:uid="{2A19314A-905C-4054-ADD7-A1EBA22B0614}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D08D0399-882A-448B-957D-AEDB0D78416D}" name="tbParcelamentos" displayName="tbParcelamentos" ref="A1:G2" totalsRowShown="0">
+  <autoFilter ref="A1:G2" xr:uid="{D08D0399-882A-448B-957D-AEDB0D78416D}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B692F6B1-C598-4022-9E71-E0C28D5660B3}" name="Compra"/>
+    <tableColumn id="2" xr3:uid="{D3B96191-9482-4F00-BAA1-1378B31F8D65}" name="Cartao"/>
+    <tableColumn id="3" xr3:uid="{7BB38C14-985D-4CEA-A1ED-EF9A0E6C6243}" name="Parcela_Atual"/>
+    <tableColumn id="4" xr3:uid="{26EFF008-2EE6-4390-8FF4-2DC15A60771C}" name="Total_Parcelas"/>
+    <tableColumn id="5" xr3:uid="{9C04B655-8FA0-44E8-9532-A526F1A93A1A}" name="Valor_Parcela" dataCellStyle="Moeda">
+      <calculatedColumnFormula>3000/10</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{14BFBE8A-3882-4A32-8833-7FACBD156179}" name="Competencia"/>
+    <tableColumn id="7" xr3:uid="{15B21A92-783D-4790-9C59-6F554DA4A226}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}" name="tbConfiguracoes" displayName="tbConfiguracoes" ref="A1:B7" totalsRowShown="0">
   <autoFilter ref="A1:B7" xr:uid="{678C3B75-1E22-47EE-AB6E-47AFD03B2FC6}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{D2936EAB-86F0-4B66-ACE9-63DAD986A44F}" name="Parametro"/>
     <tableColumn id="2" xr3:uid="{F4458E02-E9B4-48E4-A708-C914B6098752}" name="Valor"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{83676618-628E-4768-825A-99B3A899E190}" name="tbFaturas" displayName="tbFaturas" ref="A1:E2" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{83676618-628E-4768-825A-99B3A899E190}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{0AF3881D-039C-450F-BDF3-B1AD9DA17C3C}" name="Cartao"/>
+    <tableColumn id="2" xr3:uid="{FA79969F-378E-465F-9FA2-2DC15083FF25}" name="Competencia"/>
+    <tableColumn id="3" xr3:uid="{635B54C2-B09C-4219-9388-98913CE16273}" name="Data_Vencimento"/>
+    <tableColumn id="4" xr3:uid="{76B3FB2C-50C7-401A-8FAF-C0A994F26EE4}" name="Valor_Fatura" dataCellStyle="Moeda"/>
+    <tableColumn id="5" xr3:uid="{C333E680-2E35-4A3C-B283-898308283221}" name="Status_Pagamento"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D108D5BF-5273-4DD3-BF34-DAF15B1BC9CB}" name="tbLancamentosCartao" displayName="tbLancamentosCartao" ref="A1:G3" totalsRowShown="0">
+  <autoFilter ref="A1:G3" xr:uid="{D108D5BF-5273-4DD3-BF34-DAF15B1BC9CB}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{300FC87F-80AC-4FA7-891F-5E3FA9A6FB00}" name="Data_Compra"/>
+    <tableColumn id="2" xr3:uid="{0F3868B5-5AE6-43F4-842F-B4A60C339036}" name="Cartao"/>
+    <tableColumn id="3" xr3:uid="{80D163FC-B750-4A49-BAD3-68C117C26A17}" name="Descricao"/>
+    <tableColumn id="4" xr3:uid="{92513AD5-BC98-4567-AFF0-8B2687B3D2E2}" name="Categoria"/>
+    <tableColumn id="5" xr3:uid="{844181EA-79A8-48F8-96D5-20F9841C58E9}" name="Valor" dataCellStyle="Moeda"/>
+    <tableColumn id="6" xr3:uid="{066B3341-D551-44B2-9386-B136526CD890}" name="Parcelas"/>
+    <tableColumn id="7" xr3:uid="{1D83AF99-FD53-47A8-932E-8B680DB6B858}" name="Competencia"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -736,13 +889,22 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25ADEA5B-E592-467E-96CE-CA4251B085F7}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="9" width="18.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" customWidth="1"/>
+    <col min="7" max="7" width="18.7109375" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" customWidth="1"/>
+    <col min="11" max="11" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -758,8 +920,11 @@
       <c r="I1" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K1" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -775,8 +940,11 @@
       <c r="I2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -792,8 +960,11 @@
       <c r="I3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -809,8 +980,11 @@
       <c r="I4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -826,21 +1000,30 @@
       <c r="I5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>10</v>
       </c>
       <c r="E6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="K7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>4</v>
       </c>
@@ -926,6 +1109,152 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25FC72ED-E857-46F3-96F1-3B41006EF91A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F2F6950-DF9E-449A-BF3E-C4B1FEB22D19}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="14.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="5">
+        <v>46204</v>
+      </c>
+      <c r="C2" s="2">
+        <v>46212</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1573.32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{0F47FC29-5DFE-411B-A260-1A983B6915A4}">
+      <formula1>lstCartoes</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6EDF0A3-2F5D-4F56-BA65-9B247DC5D79D}">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="3" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>46216</v>
+      </c>
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="3">
+        <v>3000</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2" s="5">
+        <v>46204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E3" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B3" xr:uid="{81F4BA1A-5476-41F4-9587-CB93B97940F3}">
+      <formula1>lstCartoes</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D3" xr:uid="{1D6A2C00-ECB4-43E5-A997-CFB1EDAA1C59}">
+      <formula1>lstCategoriasCartao</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A62F83D-97A7-4FCB-A87A-BE593C175B40}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -1157,19 +1486,193 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50634029-1690-41A0-83DB-813CACF2A824}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="3">
+        <v>5500</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="3">
+        <v>19530</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3000</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2500</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28EAEDA-7868-4003-99EF-6D6DDD98D4D1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="6" max="6" width="14.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2" s="3">
+        <f>3000/10</f>
+        <v>300</v>
+      </c>
+      <c r="F2" s="5">
+        <v>46204</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{D48BF84F-49C1-4D0D-B21F-17B1E9CC45C8}">
+      <formula1>lstStatus</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Cria estrutura inicial de parcelamentos
</commit_message>
<xml_diff>
--- a/Sistema_Financeiro_Carlos_v1.xlsx
+++ b/Sistema_Financeiro_Carlos_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos.renato\meu-primeiro-repositorio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6FEC1B3-8803-45FF-A9FA-4BC6FFF63069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16DE0733-6ED1-4D76-A99C-0376B9EA86F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" firstSheet="10" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -86,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="85">
   <si>
     <t>Tipos_Receita</t>
   </si>
@@ -335,6 +335,12 @@
   </si>
   <si>
     <t>Valor_Parcela</t>
+  </si>
+  <si>
+    <t>ID_Compra</t>
+  </si>
+  <si>
+    <t>COMP001</t>
   </si>
 </sst>
 </file>
@@ -490,9 +496,9 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D08D0399-882A-448B-957D-AEDB0D78416D}" name="tbParcelamentos" displayName="tbParcelamentos" ref="A1:G2" totalsRowShown="0">
-  <autoFilter ref="A1:G2" xr:uid="{D08D0399-882A-448B-957D-AEDB0D78416D}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D08D0399-882A-448B-957D-AEDB0D78416D}" name="tbParcelamentos" displayName="tbParcelamentos" ref="A1:H2" totalsRowShown="0">
+  <autoFilter ref="A1:H2" xr:uid="{D08D0399-882A-448B-957D-AEDB0D78416D}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{B692F6B1-C598-4022-9E71-E0C28D5660B3}" name="Compra"/>
     <tableColumn id="2" xr3:uid="{D3B96191-9482-4F00-BAA1-1378B31F8D65}" name="Cartao"/>
     <tableColumn id="3" xr3:uid="{7BB38C14-985D-4CEA-A1ED-EF9A0E6C6243}" name="Parcela_Atual"/>
@@ -502,6 +508,7 @@
     </tableColumn>
     <tableColumn id="6" xr3:uid="{14BFBE8A-3882-4A32-8833-7FACBD156179}" name="Competencia"/>
     <tableColumn id="7" xr3:uid="{15B21A92-783D-4790-9C59-6F554DA4A226}" name="Status"/>
+    <tableColumn id="8" xr3:uid="{F6891B9B-D433-4259-B685-C760465E008A}" name="ID_Compra"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -533,9 +540,9 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D108D5BF-5273-4DD3-BF34-DAF15B1BC9CB}" name="tbLancamentosCartao" displayName="tbLancamentosCartao" ref="A1:G3" totalsRowShown="0">
-  <autoFilter ref="A1:G3" xr:uid="{D108D5BF-5273-4DD3-BF34-DAF15B1BC9CB}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D108D5BF-5273-4DD3-BF34-DAF15B1BC9CB}" name="tbLancamentosCartao" displayName="tbLancamentosCartao" ref="A1:H3" totalsRowShown="0">
+  <autoFilter ref="A1:H3" xr:uid="{D108D5BF-5273-4DD3-BF34-DAF15B1BC9CB}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{300FC87F-80AC-4FA7-891F-5E3FA9A6FB00}" name="Data_Compra"/>
     <tableColumn id="2" xr3:uid="{0F3868B5-5AE6-43F4-842F-B4A60C339036}" name="Cartao"/>
     <tableColumn id="3" xr3:uid="{80D163FC-B750-4A49-BAD3-68C117C26A17}" name="Descricao"/>
@@ -543,6 +550,7 @@
     <tableColumn id="5" xr3:uid="{844181EA-79A8-48F8-96D5-20F9841C58E9}" name="Valor" dataCellStyle="Moeda"/>
     <tableColumn id="6" xr3:uid="{066B3341-D551-44B2-9386-B136526CD890}" name="Parcelas"/>
     <tableColumn id="7" xr3:uid="{1D83AF99-FD53-47A8-932E-8B680DB6B858}" name="Competencia"/>
+    <tableColumn id="8" xr3:uid="{C059D2C4-BAD7-4B4D-8455-1263B16325EA}" name="ID_Compra"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1177,7 +1185,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6EDF0A3-2F5D-4F56-BA65-9B247DC5D79D}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1185,9 +1193,10 @@
     <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.42578125" customWidth="1"/>
     <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>70</v>
       </c>
@@ -1209,8 +1218,11 @@
       <c r="G1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46216</v>
       </c>
@@ -1232,8 +1244,11 @@
       <c r="G2" s="5">
         <v>46204</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E3" s="3"/>
     </row>
   </sheetData>
@@ -1606,17 +1621,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F28EAEDA-7868-4003-99EF-6D6DDD98D4D1}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>79</v>
       </c>
@@ -1638,8 +1654,11 @@
       <c r="G1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -1661,6 +1680,9 @@
       </c>
       <c r="G2" t="s">
         <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>